<commit_message>
Spreadsheets: FILTER without Excel prefix, Leia-me text kept as text
Google Sheets rejects _xlfn._xlws.FILTER, and Leia-me lines starting with '='
were imported as broken formulas; '*' inside formulas is no longer stripped.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/infobasica/planilhas/aula05_nivel1.xlsx
+++ b/assets/infobasica/planilhas/aula05_nivel1.xlsx
@@ -503,7 +503,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Largura em A2 (4,5) e comprimento em B2 (3,2); em C2, =A2B2 calcula a área.</t>
+          <t>Largura em A2 (4,5) e comprimento em B2 (3,2); em C2, =A2*B2 calcula a área.</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Para abrir no Google Planilhas: Google Drive → Novo → Upload de arquivo; depois clique no arquivo → Abrir com → Planilhas Google.</t>
+          <t>Esta é a sua cópia: altere à vontade.</t>
         </is>
       </c>
     </row>

</xml_diff>